<commit_message>
feat: increase prisma transaction timeout to 30 minutes
</commit_message>
<xml_diff>
--- a/apps/web/test-data.xlsx
+++ b/apps/web/test-data.xlsx
@@ -1,10 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B8CB8E6-72FA-4F16-9E57-7EFA9AF6BF7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Products" state="visible" r:id="rId4"/>
+    <sheet name="Products" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -49,9 +53,7 @@
     <t>TEST-HVS-A4-80</t>
   </si>
   <si>
-    <r>
-      <t>Kertas</t>
-    </r>
+    <t>Kertas</t>
   </si>
   <si>
     <t>rim</t>
@@ -75,9 +77,7 @@
     <t>TEST-PULPEN-GEL-05</t>
   </si>
   <si>
-    <r>
-      <t>Alat Tulis</t>
-    </r>
+    <t>Alat Tulis</t>
   </si>
   <si>
     <t>pcs</t>
@@ -98,9 +98,7 @@
     <t>TEST-TINTA-EPSON-BK</t>
   </si>
   <si>
-    <r>
-      <t>Tinta &amp; Cartridge</t>
-    </r>
+    <t>Tinta &amp; Cartridge</t>
   </si>
   <si>
     <t>botol</t>
@@ -127,14 +125,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -497,11 +495,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.85546875" customWidth="1"/>
+    <col min="2" max="2" width="31.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -533,7 +535,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -565,7 +567,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -597,7 +599,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -629,7 +631,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>32</v>
       </c>
@@ -662,5 +664,6 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>